<commit_message>
Add bookmarklet busy-state UI and a JSON import fallback
The Portal Reader bookmarklet now shows a spinner and elapsed-time
readout instead of static text during a scrape/commit, so a slow
portal or large batch doesn't read as frozen. When a portal's CSP
blocks the bookmarklet's direct connection to the Hub, its downloaded
.json fallback file can now be dropped into the normal import
dropzone, which routes it through /api/import/portal instead of the
.xlsx path.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Departmental/tenant_consolidated_long_budget_20260827_080349.xlsx
+++ b/Departmental/tenant_consolidated_long_budget_20260827_080349.xlsx
@@ -1,21 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Idara Maliyah\Code\Istifadah Ilmiyah\Departmental\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2338E39-5E6C-42C9-98C5-8BD1F6824B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="All Budget Entries" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="189">
   <si>
     <t>Srno</t>
   </si>
@@ -587,23 +603,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -630,18 +638,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="2" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="49" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="2" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="49" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -931,28 +947,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L97"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.856" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="43.561" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="56.558" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="19.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="56.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -990,7 +1002,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1019,7 +1031,7 @@
         <v>15</v>
       </c>
       <c r="J2" s="1">
-        <v>4153.0</v>
+        <v>4153</v>
       </c>
       <c r="K2" t="s">
         <v>16</v>
@@ -1028,7 +1040,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1057,7 +1069,7 @@
         <v>20</v>
       </c>
       <c r="J3" s="1">
-        <v>1734600.0</v>
+        <v>1734600</v>
       </c>
       <c r="K3" t="s">
         <v>21</v>
@@ -1066,7 +1078,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -1078,7 +1090,7 @@
         <v>23</v>
       </c>
       <c r="J4" s="1">
-        <v>1472625.0</v>
+        <v>1472625</v>
       </c>
       <c r="K4" t="s">
         <v>24</v>
@@ -1087,7 +1099,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -1099,13 +1111,13 @@
         <v>26</v>
       </c>
       <c r="J5" s="1">
-        <v>3000000.0</v>
+        <v>3000000</v>
       </c>
       <c r="L5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -1117,13 +1129,13 @@
         <v>28</v>
       </c>
       <c r="J6" s="1">
-        <v>1200000.0</v>
+        <v>1200000</v>
       </c>
       <c r="L6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -1135,13 +1147,13 @@
         <v>30</v>
       </c>
       <c r="J7" s="1">
-        <v>10000000.0</v>
+        <v>10000000</v>
       </c>
       <c r="L7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -1153,13 +1165,13 @@
         <v>31</v>
       </c>
       <c r="J8" s="1">
-        <v>512500.0</v>
+        <v>512500</v>
       </c>
       <c r="L8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -1171,13 +1183,13 @@
         <v>33</v>
       </c>
       <c r="J9" s="1">
-        <v>1082500.0</v>
+        <v>1082500</v>
       </c>
       <c r="L9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -1189,13 +1201,13 @@
         <v>35</v>
       </c>
       <c r="J10" s="1">
-        <v>4000000.0</v>
+        <v>4000000</v>
       </c>
       <c r="L10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1207,13 +1219,13 @@
         <v>36</v>
       </c>
       <c r="J11" s="1">
-        <v>1053300.0</v>
+        <v>1053300</v>
       </c>
       <c r="L11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>3</v>
       </c>
@@ -1238,7 +1250,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4</v>
       </c>
@@ -1263,7 +1275,7 @@
       <c r="I13" s="2"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1292,7 +1304,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="1">
-        <v>12500.0</v>
+        <v>12500</v>
       </c>
       <c r="K14" t="s">
         <v>42</v>
@@ -1301,7 +1313,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -1313,7 +1325,7 @@
         <v>43</v>
       </c>
       <c r="J15" s="1">
-        <v>12000.0</v>
+        <v>12000</v>
       </c>
       <c r="K15" t="s">
         <v>42</v>
@@ -1322,7 +1334,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -1334,7 +1346,7 @@
         <v>45</v>
       </c>
       <c r="J16" s="1">
-        <v>742118.0</v>
+        <v>742118</v>
       </c>
       <c r="K16" t="s">
         <v>46</v>
@@ -1343,7 +1355,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -1355,7 +1367,7 @@
         <v>28</v>
       </c>
       <c r="J17" s="1">
-        <v>1449393.0</v>
+        <v>1449393</v>
       </c>
       <c r="K17" t="s">
         <v>48</v>
@@ -1364,7 +1376,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -1376,7 +1388,7 @@
         <v>50</v>
       </c>
       <c r="J18" s="1">
-        <v>352820.0</v>
+        <v>352820</v>
       </c>
       <c r="K18" t="s">
         <v>51</v>
@@ -1385,7 +1397,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -1397,7 +1409,7 @@
         <v>52</v>
       </c>
       <c r="J19" s="1">
-        <v>18320.0</v>
+        <v>18320</v>
       </c>
       <c r="K19" t="s">
         <v>53</v>
@@ -1406,7 +1418,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -1418,7 +1430,7 @@
         <v>55</v>
       </c>
       <c r="J20" s="1">
-        <v>133706.0</v>
+        <v>133706</v>
       </c>
       <c r="K20" t="s">
         <v>56</v>
@@ -1427,7 +1439,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
@@ -1439,7 +1451,7 @@
         <v>57</v>
       </c>
       <c r="J21" s="1">
-        <v>48000.0</v>
+        <v>48000</v>
       </c>
       <c r="K21" t="s">
         <v>58</v>
@@ -1448,7 +1460,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
@@ -1460,7 +1472,7 @@
         <v>59</v>
       </c>
       <c r="J22" s="1">
-        <v>48000.0</v>
+        <v>48000</v>
       </c>
       <c r="K22" t="s">
         <v>58</v>
@@ -1469,7 +1481,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -1481,7 +1493,7 @@
         <v>61</v>
       </c>
       <c r="J23" s="1">
-        <v>60500.0</v>
+        <v>60500</v>
       </c>
       <c r="K23" t="s">
         <v>62</v>
@@ -1490,7 +1502,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:12">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -1502,7 +1514,7 @@
         <v>64</v>
       </c>
       <c r="J24" s="1">
-        <v>8624.0</v>
+        <v>8624</v>
       </c>
       <c r="K24" t="s">
         <v>62</v>
@@ -1511,7 +1523,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
@@ -1523,7 +1535,7 @@
         <v>65</v>
       </c>
       <c r="J25" s="1">
-        <v>7488.0</v>
+        <v>7488</v>
       </c>
       <c r="K25" t="s">
         <v>66</v>
@@ -1532,7 +1544,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -1544,7 +1556,7 @@
         <v>67</v>
       </c>
       <c r="J26" s="1">
-        <v>124801.0</v>
+        <v>124801</v>
       </c>
       <c r="K26" t="s">
         <v>56</v>
@@ -1553,7 +1565,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -1565,7 +1577,7 @@
         <v>68</v>
       </c>
       <c r="J27" s="1">
-        <v>74617.0</v>
+        <v>74617</v>
       </c>
       <c r="K27" t="s">
         <v>69</v>
@@ -1574,7 +1586,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -1586,7 +1598,7 @@
         <v>70</v>
       </c>
       <c r="J28" s="1">
-        <v>70564.0</v>
+        <v>70564</v>
       </c>
       <c r="K28" t="s">
         <v>71</v>
@@ -1595,7 +1607,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -1607,7 +1619,7 @@
         <v>73</v>
       </c>
       <c r="J29" s="1">
-        <v>36934.0</v>
+        <v>36934</v>
       </c>
       <c r="K29" t="s">
         <v>74</v>
@@ -1616,7 +1628,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -1628,13 +1640,13 @@
         <v>76</v>
       </c>
       <c r="J30" s="1">
-        <v>181971.0</v>
+        <v>181971</v>
       </c>
       <c r="L30" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -1646,13 +1658,13 @@
         <v>78</v>
       </c>
       <c r="J31" s="1">
-        <v>350000.0</v>
+        <v>350000</v>
       </c>
       <c r="L31" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>6</v>
       </c>
@@ -1681,7 +1693,7 @@
         <v>81</v>
       </c>
       <c r="J32" s="1">
-        <v>400000.0</v>
+        <v>400000</v>
       </c>
       <c r="K32" t="s">
         <v>69</v>
@@ -1690,7 +1702,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:12">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -1702,13 +1714,13 @@
         <v>28</v>
       </c>
       <c r="J33" s="1">
-        <v>400000.0</v>
+        <v>400000</v>
       </c>
       <c r="L33" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:12">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>7</v>
       </c>
@@ -1737,7 +1749,7 @@
         <v>85</v>
       </c>
       <c r="J34" s="1">
-        <v>1416000.0</v>
+        <v>1416000</v>
       </c>
       <c r="K34" t="s">
         <v>86</v>
@@ -1746,7 +1758,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -1758,13 +1770,13 @@
         <v>88</v>
       </c>
       <c r="J35" s="1">
-        <v>15000.0</v>
+        <v>15000</v>
       </c>
       <c r="L35" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:12">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -1776,13 +1788,13 @@
         <v>89</v>
       </c>
       <c r="J36" s="1">
-        <v>15263118.0</v>
+        <v>15263118</v>
       </c>
       <c r="L36" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:12">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
@@ -1794,13 +1806,13 @@
         <v>91</v>
       </c>
       <c r="J37" s="1">
-        <v>24964592.0</v>
+        <v>24964592</v>
       </c>
       <c r="L37" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -1812,13 +1824,13 @@
         <v>92</v>
       </c>
       <c r="J38" s="1">
-        <v>25000.0</v>
+        <v>25000</v>
       </c>
       <c r="L38" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="39" spans="1:12">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -1830,13 +1842,13 @@
         <v>94</v>
       </c>
       <c r="J39" s="1">
-        <v>12814465.0</v>
+        <v>12814465</v>
       </c>
       <c r="L39" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>8</v>
       </c>
@@ -1865,7 +1877,7 @@
         <v>97</v>
       </c>
       <c r="J40" s="1">
-        <v>495836.0</v>
+        <v>495836</v>
       </c>
       <c r="K40" t="s">
         <v>86</v>
@@ -1874,7 +1886,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="1:12">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
@@ -1886,13 +1898,13 @@
         <v>99</v>
       </c>
       <c r="J41" s="1">
-        <v>6000000.0</v>
+        <v>6000000</v>
       </c>
       <c r="L41" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="42" spans="1:12">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -1904,13 +1916,13 @@
         <v>88</v>
       </c>
       <c r="J42" s="1">
-        <v>4000000.0</v>
+        <v>4000000</v>
       </c>
       <c r="L42" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="43" spans="1:12">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
@@ -1922,13 +1934,13 @@
         <v>101</v>
       </c>
       <c r="J43" s="1">
-        <v>1500000.0</v>
+        <v>1500000</v>
       </c>
       <c r="L43" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="44" spans="1:12">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>9</v>
       </c>
@@ -1953,7 +1965,7 @@
       <c r="I44" s="2"/>
       <c r="J44" s="1"/>
     </row>
-    <row r="45" spans="1:12">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>10</v>
       </c>
@@ -1982,7 +1994,7 @@
         <v>70</v>
       </c>
       <c r="J45" s="1">
-        <v>9750.0</v>
+        <v>9750</v>
       </c>
       <c r="K45" t="s">
         <v>105</v>
@@ -1991,7 +2003,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:12">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -2003,7 +2015,7 @@
         <v>106</v>
       </c>
       <c r="J46" s="1">
-        <v>4700.0</v>
+        <v>4700</v>
       </c>
       <c r="K46" t="s">
         <v>107</v>
@@ -2012,7 +2024,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:12">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -2024,7 +2036,7 @@
         <v>108</v>
       </c>
       <c r="J47" s="1">
-        <v>8000.0</v>
+        <v>8000</v>
       </c>
       <c r="K47" t="s">
         <v>107</v>
@@ -2033,7 +2045,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="48" spans="1:12">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -2045,7 +2057,7 @@
         <v>109</v>
       </c>
       <c r="J48" s="1">
-        <v>8400.0</v>
+        <v>8400</v>
       </c>
       <c r="K48" t="s">
         <v>107</v>
@@ -2054,7 +2066,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="1:12">
+    <row r="49" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -2066,7 +2078,7 @@
         <v>110</v>
       </c>
       <c r="J49" s="1">
-        <v>8650.0</v>
+        <v>8650</v>
       </c>
       <c r="K49" t="s">
         <v>48</v>
@@ -2075,7 +2087,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="1:12">
+    <row r="50" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
@@ -2087,7 +2099,7 @@
         <v>111</v>
       </c>
       <c r="J50" s="1">
-        <v>10200.0</v>
+        <v>10200</v>
       </c>
       <c r="K50" t="s">
         <v>112</v>
@@ -2096,7 +2108,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="1:12">
+    <row r="51" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
@@ -2108,7 +2120,7 @@
         <v>113</v>
       </c>
       <c r="J51" s="1">
-        <v>17850.0</v>
+        <v>17850</v>
       </c>
       <c r="K51" t="s">
         <v>16</v>
@@ -2117,7 +2129,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="1:12">
+    <row r="52" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D52" s="1"/>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
@@ -2129,7 +2141,7 @@
         <v>114</v>
       </c>
       <c r="J52" s="1">
-        <v>25700.0</v>
+        <v>25700</v>
       </c>
       <c r="K52" t="s">
         <v>16</v>
@@ -2138,7 +2150,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="53" spans="1:12">
+    <row r="53" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
@@ -2150,7 +2162,7 @@
         <v>115</v>
       </c>
       <c r="J53" s="1">
-        <v>15300.0</v>
+        <v>15300</v>
       </c>
       <c r="K53" t="s">
         <v>116</v>
@@ -2159,7 +2171,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="1:12">
+    <row r="54" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
@@ -2171,7 +2183,7 @@
         <v>117</v>
       </c>
       <c r="J54" s="1">
-        <v>30000.0</v>
+        <v>30000</v>
       </c>
       <c r="K54" t="s">
         <v>116</v>
@@ -2180,7 +2192,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="55" spans="1:12">
+    <row r="55" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
@@ -2192,7 +2204,7 @@
         <v>118</v>
       </c>
       <c r="J55" s="1">
-        <v>7650.0</v>
+        <v>7650</v>
       </c>
       <c r="K55" t="s">
         <v>53</v>
@@ -2201,7 +2213,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="1:12">
+    <row r="56" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
@@ -2213,7 +2225,7 @@
         <v>119</v>
       </c>
       <c r="J56" s="1">
-        <v>32700.0</v>
+        <v>32700</v>
       </c>
       <c r="K56" t="s">
         <v>53</v>
@@ -2222,7 +2234,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:12">
+    <row r="57" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D57" s="1"/>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
@@ -2234,7 +2246,7 @@
         <v>120</v>
       </c>
       <c r="J57" s="1">
-        <v>22300.0</v>
+        <v>22300</v>
       </c>
       <c r="K57" t="s">
         <v>53</v>
@@ -2243,7 +2255,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:12">
+    <row r="58" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
@@ -2255,7 +2267,7 @@
         <v>121</v>
       </c>
       <c r="J58" s="1">
-        <v>196965.0</v>
+        <v>196965</v>
       </c>
       <c r="K58" t="s">
         <v>56</v>
@@ -2264,7 +2276,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:12">
+    <row r="59" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
@@ -2276,7 +2288,7 @@
         <v>123</v>
       </c>
       <c r="J59" s="1">
-        <v>12980.0</v>
+        <v>12980</v>
       </c>
       <c r="K59" t="s">
         <v>56</v>
@@ -2285,7 +2297,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="60" spans="1:12">
+    <row r="60" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D60" s="1"/>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
@@ -2297,7 +2309,7 @@
         <v>125</v>
       </c>
       <c r="J60" s="1">
-        <v>445680.0</v>
+        <v>445680</v>
       </c>
       <c r="K60" t="s">
         <v>66</v>
@@ -2306,7 +2318,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="61" spans="1:12">
+    <row r="61" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
@@ -2318,7 +2330,7 @@
         <v>127</v>
       </c>
       <c r="J61" s="1">
-        <v>15500.0</v>
+        <v>15500</v>
       </c>
       <c r="K61" t="s">
         <v>56</v>
@@ -2327,7 +2339,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="62" spans="1:12">
+    <row r="62" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
@@ -2339,7 +2351,7 @@
         <v>128</v>
       </c>
       <c r="J62" s="1">
-        <v>200000.0</v>
+        <v>200000</v>
       </c>
       <c r="K62" t="s">
         <v>66</v>
@@ -2348,7 +2360,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="63" spans="1:12">
+    <row r="63" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
@@ -2360,7 +2372,7 @@
         <v>129</v>
       </c>
       <c r="J63" s="1">
-        <v>125820.0</v>
+        <v>125820</v>
       </c>
       <c r="K63" t="s">
         <v>58</v>
@@ -2369,7 +2381,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="64" spans="1:12">
+    <row r="64" spans="4:12" x14ac:dyDescent="0.25">
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
@@ -2381,7 +2393,7 @@
         <v>130</v>
       </c>
       <c r="J64" s="1">
-        <v>121820.0</v>
+        <v>121820</v>
       </c>
       <c r="K64" t="s">
         <v>58</v>
@@ -2390,7 +2402,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
@@ -2402,7 +2414,7 @@
         <v>131</v>
       </c>
       <c r="J65" s="1">
-        <v>506200.0</v>
+        <v>506200</v>
       </c>
       <c r="K65" t="s">
         <v>132</v>
@@ -2411,7 +2423,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
@@ -2423,7 +2435,7 @@
         <v>133</v>
       </c>
       <c r="J66" s="1">
-        <v>1034225.0</v>
+        <v>1034225</v>
       </c>
       <c r="K66" t="s">
         <v>132</v>
@@ -2432,7 +2444,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D67" s="1"/>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
@@ -2444,7 +2456,7 @@
         <v>135</v>
       </c>
       <c r="J67" s="1">
-        <v>117100.0</v>
+        <v>117100</v>
       </c>
       <c r="K67" t="s">
         <v>24</v>
@@ -2453,7 +2465,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D68" s="1"/>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
@@ -2465,7 +2477,7 @@
         <v>136</v>
       </c>
       <c r="J68" s="1">
-        <v>18000.0</v>
+        <v>18000</v>
       </c>
       <c r="K68" t="s">
         <v>24</v>
@@ -2474,7 +2486,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
@@ -2486,13 +2498,13 @@
         <v>35</v>
       </c>
       <c r="J69" s="1">
-        <v>1000000.0</v>
+        <v>1000000</v>
       </c>
       <c r="L69" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>11</v>
       </c>
@@ -2517,7 +2529,7 @@
       <c r="I70" s="2"/>
       <c r="J70" s="1"/>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>12</v>
       </c>
@@ -2542,7 +2554,7 @@
       <c r="I71" s="2"/>
       <c r="J71" s="1"/>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>13</v>
       </c>
@@ -2571,7 +2583,7 @@
         <v>141</v>
       </c>
       <c r="J72" s="1">
-        <v>29625.0</v>
+        <v>29625</v>
       </c>
       <c r="K72" t="s">
         <v>16</v>
@@ -2580,7 +2592,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D73" s="1"/>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
@@ -2592,7 +2604,7 @@
         <v>129</v>
       </c>
       <c r="J73" s="1">
-        <v>5100.0</v>
+        <v>5100</v>
       </c>
       <c r="K73" t="s">
         <v>53</v>
@@ -2601,7 +2613,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
@@ -2613,7 +2625,7 @@
         <v>130</v>
       </c>
       <c r="J74" s="1">
-        <v>54250.0</v>
+        <v>54250</v>
       </c>
       <c r="K74" t="s">
         <v>53</v>
@@ -2622,7 +2634,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D75" s="1"/>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
@@ -2634,7 +2646,7 @@
         <v>143</v>
       </c>
       <c r="J75" s="1">
-        <v>21000.0</v>
+        <v>21000</v>
       </c>
       <c r="K75" t="s">
         <v>144</v>
@@ -2643,7 +2655,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" spans="1:12">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D76" s="1"/>
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
@@ -2655,7 +2667,7 @@
         <v>50</v>
       </c>
       <c r="J76" s="1">
-        <v>8086.0</v>
+        <v>8086</v>
       </c>
       <c r="K76" t="s">
         <v>145</v>
@@ -2664,7 +2676,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="77" spans="1:12">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D77" s="1"/>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
@@ -2676,7 +2688,7 @@
         <v>147</v>
       </c>
       <c r="J77" s="1">
-        <v>124677.0</v>
+        <v>124677</v>
       </c>
       <c r="K77" t="s">
         <v>74</v>
@@ -2685,7 +2697,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="78" spans="1:12">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D78" s="1"/>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
@@ -2697,7 +2709,7 @@
         <v>149</v>
       </c>
       <c r="J78" s="1">
-        <v>287100.0</v>
+        <v>287100</v>
       </c>
       <c r="K78" t="s">
         <v>24</v>
@@ -2706,7 +2718,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="79" spans="1:12">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D79" s="1"/>
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
@@ -2718,13 +2730,13 @@
         <v>150</v>
       </c>
       <c r="J79" s="1">
-        <v>510000.0</v>
+        <v>510000</v>
       </c>
       <c r="L79" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="80" spans="1:12">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
@@ -2736,13 +2748,13 @@
         <v>152</v>
       </c>
       <c r="J80" s="1">
-        <v>650000.0</v>
+        <v>650000</v>
       </c>
       <c r="L80" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="81" spans="1:12">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D81" s="1"/>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
@@ -2754,13 +2766,13 @@
         <v>154</v>
       </c>
       <c r="J81" s="1">
-        <v>1200000.0</v>
+        <v>1200000</v>
       </c>
       <c r="L81" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="82" spans="1:12">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>14</v>
       </c>
@@ -2789,7 +2801,7 @@
         <v>157</v>
       </c>
       <c r="J82" s="1">
-        <v>185900.0</v>
+        <v>185900</v>
       </c>
       <c r="K82" t="s">
         <v>158</v>
@@ -2798,7 +2810,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="83" spans="1:12">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D83" s="1"/>
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
@@ -2810,7 +2822,7 @@
         <v>160</v>
       </c>
       <c r="J83" s="1">
-        <v>2250.0</v>
+        <v>2250</v>
       </c>
       <c r="K83" t="s">
         <v>161</v>
@@ -2819,7 +2831,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="84" spans="1:12">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D84" s="1"/>
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
@@ -2831,7 +2843,7 @@
         <v>162</v>
       </c>
       <c r="J84" s="1">
-        <v>35001.0</v>
+        <v>35001</v>
       </c>
       <c r="K84" t="s">
         <v>161</v>
@@ -2840,7 +2852,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="85" spans="1:12">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D85" s="1"/>
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
@@ -2852,7 +2864,7 @@
         <v>163</v>
       </c>
       <c r="J85" s="1">
-        <v>21561.0</v>
+        <v>21561</v>
       </c>
       <c r="K85" t="s">
         <v>161</v>
@@ -2861,7 +2873,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="86" spans="1:12">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D86" s="1"/>
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
@@ -2873,7 +2885,7 @@
         <v>164</v>
       </c>
       <c r="J86" s="1">
-        <v>1384.0</v>
+        <v>1384</v>
       </c>
       <c r="K86" t="s">
         <v>56</v>
@@ -2882,7 +2894,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="87" spans="1:12">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>15</v>
       </c>
@@ -2911,13 +2923,13 @@
         <v>167</v>
       </c>
       <c r="J87" s="1">
-        <v>700000.0</v>
+        <v>700000</v>
       </c>
       <c r="L87" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="88" spans="1:12">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D88" s="1"/>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
@@ -2929,13 +2941,13 @@
         <v>169</v>
       </c>
       <c r="J88" s="1">
-        <v>477000.0</v>
+        <v>477000</v>
       </c>
       <c r="L88" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="89" spans="1:12">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>16</v>
       </c>
@@ -2964,7 +2976,7 @@
         <v>172</v>
       </c>
       <c r="J89" s="1">
-        <v>161734.0</v>
+        <v>161734</v>
       </c>
       <c r="K89" t="s">
         <v>132</v>
@@ -2973,7 +2985,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="90" spans="1:12">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D90" s="1"/>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
@@ -2985,13 +2997,13 @@
         <v>174</v>
       </c>
       <c r="J90" s="1">
-        <v>1500000.0</v>
+        <v>1500000</v>
       </c>
       <c r="L90" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="91" spans="1:12">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>17</v>
       </c>
@@ -3020,13 +3032,13 @@
         <v>28</v>
       </c>
       <c r="J91" s="1">
-        <v>395000.0</v>
+        <v>395000</v>
       </c>
       <c r="L91" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="92" spans="1:12">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D92" s="1"/>
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
@@ -3038,13 +3050,13 @@
         <v>178</v>
       </c>
       <c r="J92" s="1">
-        <v>250000.0</v>
+        <v>250000</v>
       </c>
       <c r="L92" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="93" spans="1:12">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>18</v>
       </c>
@@ -3073,7 +3085,7 @@
         <v>181</v>
       </c>
       <c r="J93" s="1">
-        <v>480000.0</v>
+        <v>480000</v>
       </c>
       <c r="K93" t="s">
         <v>21</v>
@@ -3082,7 +3094,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="94" spans="1:12">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D94" s="1"/>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
@@ -3094,7 +3106,7 @@
         <v>182</v>
       </c>
       <c r="J94" s="1">
-        <v>70092.0</v>
+        <v>70092</v>
       </c>
       <c r="K94" t="s">
         <v>116</v>
@@ -3103,7 +3115,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="95" spans="1:12">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>19</v>
       </c>
@@ -3132,48 +3144,37 @@
         <v>186</v>
       </c>
       <c r="J95" s="1">
-        <v>150000.0</v>
+        <v>150000</v>
       </c>
       <c r="L95" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="97" spans="1:12">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3" t="s">
         <v>188</v>
       </c>
       <c r="D97" s="3">
-        <v>51300000.0</v>
+        <v>51300000</v>
       </c>
       <c r="E97" s="3"/>
       <c r="F97" s="3">
-        <v>106401295.0</v>
+        <v>106401295</v>
       </c>
       <c r="G97" s="3">
-        <v>-106401295.0</v>
+        <v>-106401295</v>
       </c>
       <c r="H97" s="3"/>
       <c r="I97" s="3"/>
       <c r="J97" s="3">
-        <v>106401295.0</v>
+        <v>106401295</v>
       </c>
       <c r="K97" s="3"/>
       <c r="L97" s="3"/>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>